<commit_message>
MAJ ressources excel sprint ressources h + lien vers open assessemnt pour les trois rôles
</commit_message>
<xml_diff>
--- a/documents/sprint/gestion-ressources.xlsx
+++ b/documents/sprint/gestion-ressources.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wamp64\www\000-agile\documents\sprint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{40DBB49E-ADB6-480F-96E7-0056B3C393AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40677A5A-E0DB-42D4-9167-E74A9E96000E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13740" activeTab="2" xr2:uid="{240C528E-C664-4C79-A268-6A38B1567254}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{240C528E-C664-4C79-A268-6A38B1567254}"/>
   </bookViews>
   <sheets>
     <sheet name="sprint idéal" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
   <si>
     <t>Lun</t>
   </si>
@@ -122,6 +122,15 @@
   </si>
   <si>
     <t>Marco à pris 2 jours</t>
+  </si>
+  <si>
+    <t>SP validé</t>
+  </si>
+  <si>
+    <t>Sp Restant</t>
+  </si>
+  <si>
+    <t>Jour de sprint</t>
   </si>
 </sst>
 </file>
@@ -879,13 +888,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF952D0D-6B61-4439-A5C0-B16E1F83766B}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.8984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -908,7 +917,7 @@
         <v>1.8999999999999997</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -922,12 +931,137 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>26</v>
       </c>
       <c r="B4">
         <f>B2*$F1</f>
+        <v>47.499999999999993</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7">
+        <v>6</v>
+      </c>
+      <c r="I7">
+        <v>7</v>
+      </c>
+      <c r="J7">
+        <v>8</v>
+      </c>
+      <c r="K7">
+        <v>9</v>
+      </c>
+      <c r="L7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9">
+        <f>B2*$F1</f>
+        <v>47.499999999999993</v>
+      </c>
+      <c r="C9">
+        <f>$B9-C8</f>
+        <v>47.499999999999993</v>
+      </c>
+      <c r="D9">
+        <f>$B9-(SUM($C8:D8))</f>
+        <v>47.499999999999993</v>
+      </c>
+      <c r="E9">
+        <f>$B9-(SUM($C8:E8))</f>
+        <v>47.499999999999993</v>
+      </c>
+      <c r="F9">
+        <f>$B9-(SUM($C8:F8))</f>
+        <v>47.499999999999993</v>
+      </c>
+      <c r="G9">
+        <f>$B9-(SUM($C8:G8))</f>
+        <v>47.499999999999993</v>
+      </c>
+      <c r="H9">
+        <f>$B9-(SUM($C8:H8))</f>
+        <v>47.499999999999993</v>
+      </c>
+      <c r="I9">
+        <f>$B9-(SUM($C8:I8))</f>
+        <v>47.499999999999993</v>
+      </c>
+      <c r="J9">
+        <f>$B9-(SUM($C8:J8))</f>
+        <v>47.499999999999993</v>
+      </c>
+      <c r="K9">
+        <f>$B9-(SUM($C8:K8))</f>
+        <v>47.499999999999993</v>
+      </c>
+      <c r="L9">
+        <f>$B9-(SUM($C8:L8))</f>
         <v>47.499999999999993</v>
       </c>
     </row>

</xml_diff>

<commit_message>
modification fichier gestion ressource excel
</commit_message>
<xml_diff>
--- a/documents/sprint/gestion-ressources.xlsx
+++ b/documents/sprint/gestion-ressources.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wamp64\www\000-agile\documents\sprint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40677A5A-E0DB-42D4-9167-E74A9E96000E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A43AA66-1B18-42B7-B309-4ACC7886A372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{240C528E-C664-4C79-A268-6A38B1567254}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13740" xr2:uid="{240C528E-C664-4C79-A268-6A38B1567254}"/>
   </bookViews>
   <sheets>
     <sheet name="sprint idéal" sheetId="1" r:id="rId1"/>
@@ -633,7 +633,7 @@
       </c>
       <c r="K3" s="1">
         <f>8-(SUM(K4:K8))</f>
-        <v>6.25</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
@@ -738,7 +738,7 @@
         <v>0</v>
       </c>
       <c r="K6" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -773,7 +773,7 @@
         <v>0</v>
       </c>
       <c r="K7" s="8">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
@@ -808,7 +808,7 @@
         <v>0</v>
       </c>
       <c r="K8" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
@@ -825,7 +825,7 @@
       </c>
       <c r="B11" s="1">
         <f>SUM(B3:K3)</f>
-        <v>72.25</v>
+        <v>66.25</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
@@ -834,7 +834,7 @@
       </c>
       <c r="B12" s="1">
         <f>$B10*$B11</f>
-        <v>216.75</v>
+        <v>198.75</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -869,7 +869,7 @@
       </c>
       <c r="B16">
         <f>$B12/8</f>
-        <v>27.09375</v>
+        <v>24.84375</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -878,7 +878,7 @@
       </c>
       <c r="B17">
         <f>B12/B10/10</f>
-        <v>7.2249999999999996</v>
+        <v>6.625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajout modifiction temps par jour homme sur gestion ressources
</commit_message>
<xml_diff>
--- a/documents/sprint/gestion-ressources.xlsx
+++ b/documents/sprint/gestion-ressources.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wamp64\www\000-agile\documents\sprint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A43AA66-1B18-42B7-B309-4ACC7886A372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{648BB392-F660-42F7-8C0F-C04E5C8EFA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13740" xr2:uid="{240C528E-C664-4C79-A268-6A38B1567254}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="32">
   <si>
     <t>Lun</t>
   </si>
@@ -131,6 +131,9 @@
   </si>
   <si>
     <t>Jour de sprint</t>
+  </si>
+  <si>
+    <t>Durée d'un jour homme</t>
   </si>
 </sst>
 </file>
@@ -549,336 +552,344 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{321C9E21-B05A-4D28-B32C-9D5E2A03B9C5}">
-  <dimension ref="A2:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="4" max="4" width="11.8984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" t="s">
-        <v>0</v>
-      </c>
-      <c r="H2" t="s">
-        <v>1</v>
-      </c>
-      <c r="I2" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" t="s">
-        <v>4</v>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1">
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" t="s">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1</v>
+      </c>
+      <c r="I3" t="s">
+        <v>3</v>
+      </c>
+      <c r="J3" t="s">
+        <v>2</v>
+      </c>
+      <c r="K3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="1">
-        <f t="shared" ref="B3:J3" si="0">8-(SUM(B4:B8))</f>
-        <v>4</v>
-      </c>
-      <c r="C3" s="1">
+      <c r="B4" s="1">
+        <f>$B$1-(SUM(B5:B9))</f>
+        <v>5</v>
+      </c>
+      <c r="C4" s="1">
+        <f t="shared" ref="C4:K4" si="0">$B$1-(SUM(C5:C9))</f>
+        <v>6.5</v>
+      </c>
+      <c r="D4" s="1">
         <f t="shared" si="0"/>
-        <v>7.75</v>
-      </c>
-      <c r="D3" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="E4" s="1">
         <f t="shared" si="0"/>
-        <v>7.75</v>
-      </c>
-      <c r="E3" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="F4" s="1">
         <f t="shared" si="0"/>
-        <v>7.75</v>
-      </c>
-      <c r="F3" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="G4" s="1">
         <f t="shared" si="0"/>
-        <v>7.75</v>
-      </c>
-      <c r="G3" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="H4" s="1">
         <f t="shared" si="0"/>
-        <v>7.75</v>
-      </c>
-      <c r="H3" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="I4" s="1">
         <f t="shared" si="0"/>
-        <v>7.75</v>
-      </c>
-      <c r="I3" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="J4" s="1">
         <f t="shared" si="0"/>
-        <v>7.75</v>
-      </c>
-      <c r="J3" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="K4" s="1">
         <f t="shared" si="0"/>
-        <v>7.75</v>
-      </c>
-      <c r="K3" s="1">
-        <f>8-(SUM(K4:K8))</f>
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="4">
-        <v>4</v>
-      </c>
-      <c r="C4" s="4">
-        <v>0</v>
-      </c>
-      <c r="D4" s="4">
-        <v>0</v>
-      </c>
-      <c r="E4" s="4">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4">
-        <v>0</v>
-      </c>
-      <c r="G4" s="4">
-        <v>0</v>
-      </c>
-      <c r="H4" s="4">
-        <v>0</v>
-      </c>
-      <c r="I4" s="4">
-        <v>0</v>
-      </c>
-      <c r="J4" s="4">
-        <v>0</v>
-      </c>
-      <c r="K4" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="B5" s="4">
+        <v>2</v>
+      </c>
+      <c r="C5" s="4">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="6">
-        <v>0</v>
-      </c>
-      <c r="C5" s="6">
-        <v>0.25</v>
-      </c>
-      <c r="D5" s="6">
-        <v>0.25</v>
-      </c>
-      <c r="E5" s="6">
-        <v>0.25</v>
-      </c>
-      <c r="F5" s="6">
-        <v>0.25</v>
-      </c>
-      <c r="G5" s="6">
-        <v>0.25</v>
-      </c>
-      <c r="H5" s="6">
-        <v>0.25</v>
-      </c>
-      <c r="I5" s="6">
-        <v>0.25</v>
-      </c>
-      <c r="J5" s="6">
-        <v>0.25</v>
-      </c>
-      <c r="K5" s="6">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="8">
-        <v>0</v>
-      </c>
-      <c r="C6" s="8">
-        <v>0</v>
-      </c>
-      <c r="D6" s="8">
-        <v>0</v>
-      </c>
-      <c r="E6" s="8">
-        <v>0</v>
-      </c>
-      <c r="F6" s="8">
-        <v>0</v>
-      </c>
-      <c r="G6" s="8">
-        <v>0</v>
-      </c>
-      <c r="H6" s="8">
-        <v>0</v>
-      </c>
-      <c r="I6" s="8">
-        <v>0</v>
-      </c>
-      <c r="J6" s="8">
-        <v>0</v>
-      </c>
-      <c r="K6" s="8">
-        <v>2</v>
+      <c r="B6" s="6">
+        <v>0</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="D6" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="E6" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="F6" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="G6" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="H6" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="I6" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="J6" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="K6" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="8">
+        <v>0</v>
+      </c>
+      <c r="C7" s="8">
+        <v>0</v>
+      </c>
+      <c r="D7" s="8">
+        <v>0</v>
+      </c>
+      <c r="E7" s="8">
+        <v>0</v>
+      </c>
+      <c r="F7" s="8">
+        <v>0</v>
+      </c>
+      <c r="G7" s="8">
+        <v>0</v>
+      </c>
+      <c r="H7" s="8">
+        <v>0</v>
+      </c>
+      <c r="I7" s="8">
+        <v>0</v>
+      </c>
+      <c r="J7" s="8">
+        <v>0</v>
+      </c>
+      <c r="K7" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="8">
-        <v>0</v>
-      </c>
-      <c r="C7" s="8">
-        <v>0</v>
-      </c>
-      <c r="D7" s="8">
-        <v>0</v>
-      </c>
-      <c r="E7" s="8">
-        <v>0</v>
-      </c>
-      <c r="F7" s="8">
-        <v>0</v>
-      </c>
-      <c r="G7" s="8">
-        <v>0</v>
-      </c>
-      <c r="H7" s="8">
-        <v>0</v>
-      </c>
-      <c r="I7" s="8">
-        <v>0</v>
-      </c>
-      <c r="J7" s="8">
-        <v>0</v>
-      </c>
-      <c r="K7" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B8" s="8">
+        <v>0</v>
+      </c>
+      <c r="C8" s="8">
+        <v>0</v>
+      </c>
+      <c r="D8" s="8">
+        <v>0</v>
+      </c>
+      <c r="E8" s="8">
+        <v>0</v>
+      </c>
+      <c r="F8" s="8">
+        <v>0</v>
+      </c>
+      <c r="G8" s="8">
+        <v>0</v>
+      </c>
+      <c r="H8" s="8">
+        <v>0</v>
+      </c>
+      <c r="I8" s="8">
+        <v>0</v>
+      </c>
+      <c r="J8" s="8">
+        <v>0</v>
+      </c>
+      <c r="K8" s="8">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="2">
-        <v>0</v>
-      </c>
-      <c r="C8" s="2">
-        <v>0</v>
-      </c>
-      <c r="D8" s="2">
-        <v>0</v>
-      </c>
-      <c r="E8" s="2">
-        <v>0</v>
-      </c>
-      <c r="F8" s="2">
-        <v>0</v>
-      </c>
-      <c r="G8" s="2">
-        <v>0</v>
-      </c>
-      <c r="H8" s="2">
-        <v>0</v>
-      </c>
-      <c r="I8" s="2">
-        <v>0</v>
-      </c>
-      <c r="J8" s="2">
-        <v>0</v>
-      </c>
-      <c r="K8" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10">
-        <v>3</v>
+      <c r="B9" s="2">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2">
+        <v>0</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2">
+        <v>5.5</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="1">
-        <f>SUM(B3:K3)</f>
-        <v>66.25</v>
+        <v>12</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B12" s="1">
-        <f>$B10*$B11</f>
-        <v>198.75</v>
+        <f>SUM(B4:K4)</f>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13">
-        <v>1.9</v>
+        <v>13</v>
+      </c>
+      <c r="B13" s="1">
+        <f>$B11*$B12</f>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="1">
-        <f>$B13*$B10</f>
-        <v>5.6999999999999993</v>
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <v>1.9</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" s="1">
-        <f>$B14*10</f>
-        <v>56.999999999999993</v>
+        <f>$B14*$B11</f>
+        <v>1.9</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16">
-        <f>$B12/8</f>
-        <v>24.84375</v>
+        <v>16</v>
+      </c>
+      <c r="B16" s="1">
+        <f>$B15*10</f>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17">
+        <f>$B13/8</f>
+        <v>7.125</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>19</v>
       </c>
-      <c r="B17">
-        <f>B12/B10/10</f>
-        <v>6.625</v>
+      <c r="B18">
+        <f>B13/B11/10</f>
+        <v>5.7</v>
       </c>
     </row>
   </sheetData>
@@ -899,22 +910,22 @@
         <v>23</v>
       </c>
       <c r="B1">
-        <f>('sprint idéal'!$B10*10)</f>
-        <v>30</v>
+        <f>('sprint idéal'!$B11*10)</f>
+        <v>10</v>
       </c>
       <c r="C1" t="s">
         <v>24</v>
       </c>
       <c r="D1">
-        <f>'sprint idéal'!$B15</f>
-        <v>56.999999999999993</v>
+        <f>'sprint idéal'!$B16</f>
+        <v>19</v>
       </c>
       <c r="E1" t="s">
         <v>25</v>
       </c>
       <c r="F1">
         <f>$D1/$B1</f>
-        <v>1.8999999999999997</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
@@ -937,7 +948,7 @@
       </c>
       <c r="B4">
         <f>B2*$F1</f>
-        <v>47.499999999999993</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -1022,47 +1033,47 @@
       </c>
       <c r="B9">
         <f>B2*$F1</f>
-        <v>47.499999999999993</v>
+        <v>47.5</v>
       </c>
       <c r="C9">
         <f>$B9-C8</f>
-        <v>47.499999999999993</v>
+        <v>47.5</v>
       </c>
       <c r="D9">
         <f>$B9-(SUM($C8:D8))</f>
-        <v>47.499999999999993</v>
+        <v>47.5</v>
       </c>
       <c r="E9">
         <f>$B9-(SUM($C8:E8))</f>
-        <v>47.499999999999993</v>
+        <v>47.5</v>
       </c>
       <c r="F9">
         <f>$B9-(SUM($C8:F8))</f>
-        <v>47.499999999999993</v>
+        <v>47.5</v>
       </c>
       <c r="G9">
         <f>$B9-(SUM($C8:G8))</f>
-        <v>47.499999999999993</v>
+        <v>47.5</v>
       </c>
       <c r="H9">
         <f>$B9-(SUM($C8:H8))</f>
-        <v>47.499999999999993</v>
+        <v>47.5</v>
       </c>
       <c r="I9">
         <f>$B9-(SUM($C8:I8))</f>
-        <v>47.499999999999993</v>
+        <v>47.5</v>
       </c>
       <c r="J9">
         <f>$B9-(SUM($C8:J8))</f>
-        <v>47.499999999999993</v>
+        <v>47.5</v>
       </c>
       <c r="K9">
         <f>$B9-(SUM($C8:K8))</f>
-        <v>47.499999999999993</v>
+        <v>47.5</v>
       </c>
       <c r="L9">
         <f>$B9-(SUM($C8:L8))</f>
-        <v>47.499999999999993</v>
+        <v>47.5</v>
       </c>
     </row>
   </sheetData>
@@ -1083,22 +1094,22 @@
         <v>23</v>
       </c>
       <c r="B1">
-        <f>('sprint idéal'!$B10*10)</f>
-        <v>30</v>
+        <f>('sprint idéal'!$B11*10)</f>
+        <v>10</v>
       </c>
       <c r="C1" t="s">
         <v>24</v>
       </c>
       <c r="D1">
-        <f>'sprint idéal'!$B15</f>
-        <v>56.999999999999993</v>
+        <f>'sprint idéal'!$B16</f>
+        <v>19</v>
       </c>
       <c r="E1" t="s">
         <v>25</v>
       </c>
       <c r="F1">
         <f>$D1/$B1</f>
-        <v>1.8999999999999997</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajout ressource liens sprint review
</commit_message>
<xml_diff>
--- a/documents/sprint/gestion-ressources.xlsx
+++ b/documents/sprint/gestion-ressources.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wamp64\www\000-agile\documents\sprint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCFF74C8-7346-40ED-821E-032C11CA2E88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7303CC29-F3AE-483C-8EAE-43AD2152101A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29250" yWindow="360" windowWidth="22110" windowHeight="12555" xr2:uid="{240C528E-C664-4C79-A268-6A38B1567254}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13740" xr2:uid="{240C528E-C664-4C79-A268-6A38B1567254}"/>
   </bookViews>
   <sheets>
     <sheet name="sprint idéal" sheetId="1" r:id="rId1"/>
@@ -998,10 +998,10 @@
         <v>0</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1038,43 +1038,43 @@
       </c>
       <c r="C9">
         <f>$B9-C8</f>
-        <v>66.5</v>
+        <v>63.5</v>
       </c>
       <c r="D9">
         <f>$B9-(SUM($C8:D8))</f>
-        <v>66.5</v>
+        <v>62.5</v>
       </c>
       <c r="E9">
         <f>$B9-(SUM($C8:E8))</f>
-        <v>66.5</v>
+        <v>62.5</v>
       </c>
       <c r="F9">
         <f>$B9-(SUM($C8:F8))</f>
-        <v>66.5</v>
+        <v>62.5</v>
       </c>
       <c r="G9">
         <f>$B9-(SUM($C8:G8))</f>
-        <v>66.5</v>
+        <v>62.5</v>
       </c>
       <c r="H9">
         <f>$B9-(SUM($C8:H8))</f>
-        <v>66.5</v>
+        <v>62.5</v>
       </c>
       <c r="I9">
         <f>$B9-(SUM($C8:I8))</f>
-        <v>66.5</v>
+        <v>62.5</v>
       </c>
       <c r="J9">
         <f>$B9-(SUM($C8:J8))</f>
-        <v>66.5</v>
+        <v>62.5</v>
       </c>
       <c r="K9">
         <f>$B9-(SUM($C8:K8))</f>
-        <v>66.5</v>
+        <v>62.5</v>
       </c>
       <c r="L9">
         <f>$B9-(SUM($C8:L8))</f>
-        <v>66.5</v>
+        <v>62.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>